<commit_message>
Add new spiders for Kainan, Kitchen World Thailand, and Simply Different
- Implemented KainanSpider to scrape product listings and details from Kainan's website, supporting both search and listing modes.
- Created KitchenworldthailandSpider to extract product information, including pagination handling and SKU extraction.
- Developed SimplydifferentSpider to search for products based on SKUs from an Excel file, capturing product details and variants.
- Added a script to download images from an Excel file, generating a report of the download status.
- Included a sample JSON file with product data for Simply Different.
</commit_message>
<xml_diff>
--- a/sources/SAN NENG.xlsx
+++ b/sources/SAN NENG.xlsx
@@ -6230,35 +6230,31 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/wp-content/uploads/2021/09/SN2120.jpg</t>
+          <t>https://www.kainan-food.com.tw/upload/cht/product/1744_img_1.PNG</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>SN2125 CAKE MOULD W/O LID (NON-STICK)</t>
+          <t>三能 陽極活動蛋糕模(SN5002/SN5012/SN5022/SN5042)</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/product/sn2125-cake-mould-w-o-lid-non-stick/</t>
+          <t>https://www.kainan-food.com.tw/cht/productm/pageinfo-1744.html</t>
         </is>
       </c>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/wp-content/uploads/2021/09/SN2120.jpg; https://sinarhimalaya.com/wp-content/uploads/2021/09/SN2120-800x800.jpg</t>
+          <t>https://www.kainan-food.com.tw/upload/cht/product/1744_img_1.PNG; https://www.kainan-food.com.tw/upload/cht/product/1744_img_1.PNG; https://www.kainan-food.com.tw/upload/cht/product/2141_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1027_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2158_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2693_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1880_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1621_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2160_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2701_img_1.png</t>
         </is>
       </c>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="n">
-        <v>2</v>
-      </c>
-      <c r="M114" t="inlineStr">
-        <is>
-          <t>Jual SN2125 CAKE MOULD W/O LID (NON-STICK) Sinar Himalaya</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8571,6 +8567,41 @@
           <t>(DC21) &lt;6223565&gt;65x35 (ht) mm S/S SMALL "HEXAGON" SHAPE CAKE RING</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://kitchenworldthailand.com/front/template/default/assets/img/none-image.png</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Sanneng SN3315 S/S Hexogen Ring 65*35 mm. / ริงค์ทาร์ต</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://kitchenworldthailand.com/en/product/detail/2292</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>BAKEWARE</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>https://kitchenworldthailand.com/front/template/default/assets/img/none-image.png</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="n">
+        <v>1</v>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>Sanneng SN3315 S/S Hexogen Ring 65*35 mm. / ริงค์ทาร์ต - Kitchen World</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8953,33 +8984,37 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/wp-content/uploads/2021/09/SN3359.jpg</t>
+          <t>https://kitchenworldthailand.com/front/template/default/assets/img/none-image.png</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>SN3363 HEART RING 1.2mm 304 S/S</t>
+          <t>Sanneng SN3363 S/S Heart Ring 6" / ริงค์อบเค้ก ริงค์เค้ก ริงค์คัตเตอร์</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/product/sn3363-heart-ring-1-2mm-304-s-s/</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr"/>
+          <t>https://kitchenworldthailand.com/en/product/detail/5395</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>BAKEWARE</t>
+        </is>
+      </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/wp-content/uploads/2021/09/SN3359.jpg; https://sinarhimalaya.com/wp-content/uploads/2021/09/SN3359-800x800.jpg</t>
+          <t>https://kitchenworldthailand.com/front/template/default/assets/img/none-image.png; https://kitchenworldthailand.com//upload/pd/album/pic-20231010-1696919072-668.jpg; https://kitchenworldthailand.com//upload/pd/album/pic-20231010-1696919072-979.jpg; https://kitchenworldthailand.com//upload/pd/album/pic-20231010-1696919072-830.jpg</t>
         </is>
       </c>
       <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr"/>
       <c r="L169" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>Jual SN3363 HEART RING 1.2mm 304 S/S Sinar Himalaya</t>
+          <t>Sanneng SN3363 S/S Heart Ring 6" / ริงค์อบเค้ก ริงค์เค้ก ริงค์คัตเตอร์ - Kitchen World</t>
         </is>
       </c>
     </row>
@@ -9163,6 +9198,33 @@
           <t>&lt;6224801&gt; #SN33733 48x36x16Hmm S/S SMALL RECTANGLE CAKE RING (SAN NENG) (SELL BY PKT)</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://www.kainan-food.com.tw/upload/cht/product/2050_img_1.png</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>三能 SN33733白鐵長方鳳梨圈10入</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>https://www.kainan-food.com.tw/cht/productm/pageinfo-2050.html</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>https://www.kainan-food.com.tw/upload/cht/product/2050_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2050_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2059_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1657_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/3303_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2051_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2117_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/4249_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/4967_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/2791_img_1.png</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="n">
+        <v>10</v>
+      </c>
+      <c r="M173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -10703,6 +10765,33 @@
           <t>&lt;6112972&gt; SAN NENG-CHINA 364X60X43MM ALUMINIUM DOUBLE CRESCENT SHAPE TERRINE/JELLY MOULD</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>https://www.simplydifferent.in/cdn/shop/products/SN3573MousseCakeMould_Anodized_SangNeng9_300x300.png?v=1594454543</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>https://www.simplydifferent.in/products/mousse-cake-mould-anodised-copy?_pos=1&amp;_sid=45f6bfb24&amp;_ss=r&amp;variant=45124673405077</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr"/>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>https://www.simplydifferent.in/cdn/shop/products/SN3573MousseCakeMould_Anodized_SangNeng9_300x300.png?v=1594454543</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr"/>
+      <c r="L206" t="n">
+        <v>1</v>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>Mousse Cake Mould (Anodised)</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -10723,6 +10812,33 @@
       <c r="D207" t="inlineStr">
         <is>
           <t>&lt;6112973 SAN NENG-CHINA &gt;364X60X44.5MM ALUMINIUM TRIPLE CRESCENT SHAPE TERRINE/JELLY MOULD</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>https://www.simplydifferent.in/cdn/shop/products/SN3573MousseCakeMould_Anodized_SangNeng9_300x300.png?v=1594454543</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>https://www.simplydifferent.in/products/mousse-cake-mould-anodised-copy?_pos=1&amp;_sid=ccd329cc2&amp;_ss=r&amp;variant=45124673437845</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr"/>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>https://www.simplydifferent.in/cdn/shop/products/SN3573MousseCakeMould_Anodized_SangNeng9_300x300.png?v=1594454543</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr"/>
+      <c r="L207" t="n">
+        <v>1</v>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Mousse Cake Mould (Anodised)</t>
         </is>
       </c>
     </row>
@@ -12350,35 +12466,31 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/wp-content/uploads/2022/02/4104.jpg</t>
+          <t>https://www.kainan-food.com.tw/upload/cht/product/1777_img_1.PNG</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>SN4104 DOUGH SCRAPER, SST STEEL</t>
+          <t>焙蒂絲不鏽鋼麵包鋸刀(客訂商品)</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/product/sn4104-dough-scraper-sst-steel/</t>
+          <t>https://www.kainan-food.com.tw/cht/productm/pageinfo-1777.html</t>
         </is>
       </c>
       <c r="H239" t="inlineStr"/>
       <c r="I239" t="inlineStr">
         <is>
-          <t>https://sinarhimalaya.com/wp-content/uploads/2022/02/4104.jpg; https://sinarhimalaya.com/wp-content/uploads/2022/02/4104-800x800.jpg</t>
+          <t>https://www.kainan-food.com.tw/upload/cht/product/1777_img_1.PNG; https://www.kainan-food.com.tw/upload/cht/product/1777_img_1.PNG; https://www.kainan-food.com.tw/upload/cht/product/3296_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/5636_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1773_img_1.PNG; https://www.kainan-food.com.tw/upload/cht/product/5416_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1028_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1905_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/5642_img_1.png; https://www.kainan-food.com.tw/upload/cht/product/1835_img_1.PNG</t>
         </is>
       </c>
       <c r="J239" t="inlineStr"/>
       <c r="K239" t="inlineStr"/>
       <c r="L239" t="n">
-        <v>2</v>
-      </c>
-      <c r="M239" t="inlineStr">
-        <is>
-          <t>Jual SN4104 DOUGH SCRAPER, SST STEEL Sinar Himalaya</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="M239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -22032,6 +22144,37 @@
           <t>(DCWSL20) &lt;6164222&gt;53x38x28mm ALUM ROUND CUP MOULD (SAN NENG) (SELL BY PKT)</t>
         </is>
       </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>https://thumbnail.coupangcdn.com/thumbnails/remote/492x492ex/image/retail/images/66791426460812-6082c6f5-fa28-40f4-8116-0027bc45e4ed.jpg</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>SaNNeNg 三能 小蛋糕模 陽極 SN60225, 5個</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>https://www.tw.coupang.com/vp/products/471483897856009?itemId=471483897823243&amp;vendorItemId=471483897823239</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr"/>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>https://thumbnail.coupangcdn.com/thumbnails/remote/492x492ex/image/retail/images/66791426460812-6082c6f5-fa28-40f4-8116-0027bc45e4ed.jpg; https://img1a.coupangcdn.com/image2/size-icon.png; https://img1a.coupangcdn.com/image/sdp/option-table/icon_tabs_btn-right.png; https://thumbnail.coupangcdn.com/thumbnails/remote/q89/image/retail/images/85827982320691-663b678b-d251-4652-b672-ce91730c4f00.jpg; https://thumbnail.coupangcdn.com/thumbnails/remote/q89/image/retail/images/2374327965992786-5bc354dd-c7f7-4730-9c73-626c62afd9ca.jpg; https://thumbnail.coupangcdn.com/thumbnails/remote/q89/image/retail/images/325085906819413-3efd70c2-b6fd-4b35-b1cf-561b89f4c791.jpg; https://thumbnail.coupangcdn.com/thumbnails/remote/q89/image/retail/images/325089757007497-3dc7c632-40bf-45e8-ab63-5ba41756052b.jpg; https://thumbnail.coupangcdn.com/thumbnails/remote/q89/image/retail/images/325092705269823-c9fc087e-613c-4b42-a15d-880a84ea9ae6.jpg; https://thumbnail.coupangcdn.com/thumbnails/remote/q89/image/retail/images/325094065729892-b921ee64-f20f-45e3-9582-b2b5f23f985a.jpg; https://thumbnail.coupangcdn.com/thumbnails/remote/q89/image/retail/images/39074685449339-1e93323f-d668-4ede-a5aa-0f9d60ed862b.png</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr"/>
+      <c r="K424" t="inlineStr"/>
+      <c r="L424" t="n">
+        <v>10</v>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>SaNNeNg Small Cake Mold Anodized SN60225, 53 x 38 x ..., 5 unit - Cake Pans/Chiffon Cake Molds | Coupang</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -22601,6 +22744,37 @@
           <t>(WSL) 53x42mm ALUM HEMISPHERE DEEP CAKE MOULD (SELL BY PKT)</t>
         </is>
       </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/wp-content/uploads/2021/10/SN60505.jpg</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>SN60515 HALF SPHERE MOULD-DEEP (5PCS/SET)</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/product/sn60515-half-sphere-mould-deep-5pcs-set/</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr"/>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/wp-content/uploads/2021/10/SN60505.jpg; https://sinarhimalaya.com/wp-content/uploads/2021/10/SN60505-800x800.jpg</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr"/>
+      <c r="K437" t="inlineStr"/>
+      <c r="L437" t="n">
+        <v>2</v>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>Jual SN60515 HALF SPHERE MOULD-DEEP (5PCS/SET) Sinar Himalaya</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -22621,6 +22795,37 @@
       <c r="D438" t="inlineStr">
         <is>
           <t>(WSL) 70x58mm ALUM HEMISPHERE DEEP CAKE MOULD (SELL BY PKT)</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/wp-content/uploads/2021/10/SN60505.jpg</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>SN60535 HALF SPHERE MOULD-DEEP (5PCS/SET)</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/product/sn60535-half-sphere-mould-deep-5pcs-set/</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr"/>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/wp-content/uploads/2021/10/SN60505.jpg; https://sinarhimalaya.com/wp-content/uploads/2021/10/SN60505-800x800.jpg</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr"/>
+      <c r="K438" t="inlineStr"/>
+      <c r="L438" t="n">
+        <v>2</v>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>Jual SN60535 HALF SPHERE MOULD-DEEP (5PCS/SET) Sinar Himalaya</t>
         </is>
       </c>
     </row>
@@ -22746,6 +22951,37 @@
           <t>(DC21) &lt;6164900&gt;70x22mm "STAR" SHAPE CAKE MOULD (SELL BY PKT)</t>
         </is>
       </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/wp-content/uploads/2021/10/SN61025.jpg</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>SN61025 STAR MOULD (5PCS/SET)</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/product/sn61025-star-mould-5pcs-set/</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr"/>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>https://sinarhimalaya.com/wp-content/uploads/2021/10/SN61025.jpg; https://sinarhimalaya.com/wp-content/uploads/2021/10/SN61025-800x800.jpg</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr"/>
+      <c r="K442" t="inlineStr"/>
+      <c r="L442" t="n">
+        <v>2</v>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>Jual SN61025 STAR MOULD (5PCS/SET) Sinar Himalaya</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">

</xml_diff>